<commit_message>
corregido modulo de programas filtro y orden y creacion de plantilla programas, corregido carga masiva: se bloquean datos fantasma plantilla personalizada, corexion bug sidebar, correccion bug envio correos recuperacion de cuenta
</commit_message>
<xml_diff>
--- a/public/assets/templates/Plantilla.xlsx
+++ b/public/assets/templates/Plantilla.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
   <si>
     <t>Tipo_Documento</t>
   </si>
@@ -67,6 +67,9 @@
     <t>m.ramirez@fesc.edu.co</t>
   </si>
   <si>
+    <t>Egresado</t>
+  </si>
+  <si>
     <t>TI</t>
   </si>
   <si>
@@ -100,6 +103,9 @@
     <t>Administrativo</t>
   </si>
   <si>
+    <t>Otro</t>
+  </si>
+  <si>
     <t>PASAPORTE</t>
   </si>
   <si>
@@ -124,49 +130,7 @@
     <t>d.ortega@fesc.edu.co</t>
   </si>
   <si>
-    <t>Egresado</t>
-  </si>
-  <si>
-    <t>Kevin Jose</t>
-  </si>
-  <si>
-    <t>Duarte</t>
-  </si>
-  <si>
-    <t>k.duarte@fesc.edu.co</t>
-  </si>
-  <si>
-    <t>Sandra Lucia</t>
-  </si>
-  <si>
-    <t>Peña</t>
-  </si>
-  <si>
-    <t>s.pena@fesc.edu.co</t>
-  </si>
-  <si>
-    <t>Invitado</t>
-  </si>
-  <si>
-    <t>Otro</t>
-  </si>
-  <si>
-    <t>Ricardo Leon</t>
-  </si>
-  <si>
-    <t>Ortiz</t>
-  </si>
-  <si>
-    <t>r.ortiz@fesc.edu.co</t>
-  </si>
-  <si>
-    <t>Claudia Elena</t>
-  </si>
-  <si>
-    <t>Mejia</t>
-  </si>
-  <si>
-    <t>c.mejia@fesc.edu.co</t>
+    <t/>
   </si>
 </sst>
 </file>
@@ -174,7 +138,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -191,6 +155,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -222,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -233,20 +203,23 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -556,19 +529,19 @@
   <dimension ref="A1:J16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="9" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="9" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="9" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="10" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,12 +569,12 @@
       <c r="I1" s="3"/>
       <c r="J1" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="5">
-        <v>1090111222</v>
+        <v>1090501419</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>9</v>
@@ -616,7 +589,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="5">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>13</v>
@@ -624,7 +597,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -641,10 +614,10 @@
         <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G3" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>13</v>
@@ -652,77 +625,77 @@
       <c r="I3" s="3"/>
       <c r="J3" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4" s="5">
         <v>1090555666</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" s="5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="5">
         <v>1090777888</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" s="5">
         <v>99</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B6" s="5">
         <v>1090999000</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>12</v>
@@ -731,207 +704,191 @@
         <v>1</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" s="5">
         <v>88222333</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="G7" s="5">
         <v>2</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="5">
-        <v>1091222333</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="5">
-        <v>6</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>13</v>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5">
-        <v>1091444555</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="5">
-        <v>99</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>44</v>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="5">
-        <v>1091666777</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="5">
-        <v>3</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>22</v>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
-      <c r="A11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="5">
-        <v>1091888999</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="5">
-        <v>4</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>22</v>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" s="5"/>
+      <c r="H11" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="3"/>
-      <c r="B12" s="6"/>
+      <c r="B12" s="7"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="6"/>
+      <c r="G12" s="7"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="3"/>
-      <c r="B13" s="6"/>
+      <c r="B13" s="7"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="6"/>
+      <c r="G13" s="7"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="3"/>
-      <c r="B14" s="6"/>
+      <c r="B14" s="7"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="6"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="3"/>
-      <c r="B15" s="6"/>
+      <c r="B15" s="7"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="6"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="3"/>
-      <c r="B16" s="6"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="6"/>
+      <c r="G16" s="7"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="1"/>

</xml_diff>

<commit_message>
plataforma terminada e su version2 - fix: desactivar y activar usuarios por superadmin, se reo el cron:backup para enviar copias de seguridad en el servidor-queda pendiente programar cada seman en el servidor y config acceso a bd del server
</commit_message>
<xml_diff>
--- a/public/assets/templates/Plantilla.xlsx
+++ b/public/assets/templates/Plantilla.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t>Tipo_Documento</t>
   </si>
@@ -31,6 +31,9 @@
     <t>Correo</t>
   </si>
   <si>
+    <t>telefono</t>
+  </si>
+  <si>
     <t>Comunidad</t>
   </si>
   <si>
@@ -128,9 +131,6 @@
   </si>
   <si>
     <t>d.ortega@fesc.edu.co</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -138,7 +138,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,12 +150,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -192,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -209,10 +203,16 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -526,22 +526,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="10" width="13.005" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="12" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,338 +561,310 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3"/>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
       <c r="J1" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="5">
+      <c r="K1" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="2">
         <v>1090501419</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="5">
+        <v>3124475175</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="6">
+        <v>26</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="5"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="5">
+      <c r="B3" s="2">
+        <v>1090333444</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="7">
+        <v>4</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="K3" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1090555666</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="2">
+        <v>3</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1090777888</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="5">
-        <v>1090333444</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="5">
-        <v>4</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="5">
-        <v>1090555666</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="5">
-        <v>3</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="5">
-        <v>1090777888</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="E5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="5">
+      <c r="F5" s="4"/>
+      <c r="G5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="5">
         <v>99</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="I5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="5">
         <v>1090999000</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="5">
+      <c r="E6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="2">
         <v>1</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="I6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="2">
         <v>88222333</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="C7" s="3" t="s">
         <v>36</v>
       </c>
+      <c r="D7" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="E7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="5">
+        <v>38</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="2">
         <v>2</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="6" t="s">
-        <v>38</v>
-      </c>
+      <c r="I7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="5"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="1"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+      <c r="A9" s="3"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+      <c r="A10" s="4"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+      <c r="A11" s="3"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="6"/>
       <c r="I11" s="3"/>
       <c r="J11" s="4"/>
+      <c r="K11" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="3"/>
-      <c r="B12" s="7"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="4"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="9"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="3"/>
-      <c r="B13" s="7"/>
+      <c r="B13" s="6"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="7"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="4"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="3"/>
-      <c r="B14" s="7"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="9"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="3"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="3"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="9"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="3"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="6"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="4"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="3"/>
-      <c r="B16" s="7"/>
+      <c r="B16" s="6"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="6"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="1"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix:fomulario ivitados leyendo vista con todos los datos correspondientes - se verifica funcionamiento optimo en todo el flujo de resgistros asistencia y reporte, modulos aprobaciones y contador pendinetes corregido
</commit_message>
<xml_diff>
--- a/public/assets/templates/Plantilla.xlsx
+++ b/public/assets/templates/Plantilla.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="28">
   <si>
     <t>Tipo_Documento</t>
   </si>
@@ -40,7 +40,7 @@
     <t>ID_Prog</t>
   </si>
   <si>
-    <t>Nivel</t>
+    <t/>
   </si>
   <si>
     <t>CC</t>
@@ -58,16 +58,13 @@
     <t>Estudiante</t>
   </si>
   <si>
-    <t>Tecnólogo</t>
-  </si>
-  <si>
     <t>Maria Paula</t>
   </si>
   <si>
-    <t>Ramirez</t>
-  </si>
-  <si>
-    <t>m.ramirez@fesc.edu.co</t>
+    <t>ejemplo</t>
+  </si>
+  <si>
+    <t>ejemplo@fesc.edu.co</t>
   </si>
   <si>
     <t>Egresado</t>
@@ -79,58 +76,28 @@
     <t>Carlos Alberto</t>
   </si>
   <si>
-    <t>Gomez</t>
-  </si>
-  <si>
-    <t>c.gomez@fesc.edu.co</t>
-  </si>
-  <si>
     <t>Docente</t>
   </si>
   <si>
-    <t>Profesional</t>
-  </si>
-  <si>
     <t>CE</t>
   </si>
   <si>
     <t>Ana Milena</t>
   </si>
   <si>
-    <t>Rojas</t>
-  </si>
-  <si>
-    <t>a.rojas@fesc.edu.co</t>
-  </si>
-  <si>
     <t>Administrativo</t>
   </si>
   <si>
-    <t>Otro</t>
-  </si>
-  <si>
     <t>PASAPORTE</t>
   </si>
   <si>
     <t>Luis Fernando</t>
   </si>
   <si>
-    <t>Castro</t>
-  </si>
-  <si>
-    <t>l.castro@fesc.edu.co</t>
-  </si>
-  <si>
     <t>PPT</t>
   </si>
   <si>
     <t>Diana Marcela</t>
-  </si>
-  <si>
-    <t>Ortega</t>
-  </si>
-  <si>
-    <t>d.ortega@fesc.edu.co</t>
   </si>
 </sst>
 </file>
@@ -138,7 +105,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +122,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -186,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -194,32 +167,53 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -526,20 +520,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="10" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="11" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="12" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="16" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="17" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="16" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="16" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="16" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="16" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="17" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="16" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="16" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="19" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -558,7 +552,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -577,294 +571,291 @@
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="6">
         <v>1090501419</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="7">
         <v>3124475175</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="6">
         <v>26</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>14</v>
+      <c r="I2" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="J2" s="1"/>
-      <c r="K2" s="5"/>
+      <c r="K2" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>1090333444</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="8">
+        <v>123456789</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="10">
+        <v>4</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" s="8"/>
+      <c r="K3" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="H3" s="7">
-        <v>4</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="B4" s="2">
         <v>1090555666</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2">
+        <v>123456789</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="2">
+      <c r="H4" s="12">
         <v>3</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>24</v>
+      <c r="I4" s="13" t="s">
+        <v>8</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B5" s="2">
         <v>1090777888</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>26</v>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" s="5">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="14">
+        <v>123456789</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="2">
         <v>99</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>30</v>
+      <c r="I5" s="15" t="s">
+        <v>8</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="5">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2">
         <v>1090999000</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="5" t="s">
+      <c r="C6" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="2">
+        <v>123456789</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="8">
         <v>1</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>24</v>
+      <c r="I6" s="13" t="s">
+        <v>8</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="A7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="8">
         <v>88222333</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="1" t="s">
-        <v>18</v>
+      <c r="C7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="2">
+        <v>123456789</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="H7" s="2">
         <v>2</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>24</v>
+      <c r="I7" s="13" t="s">
+        <v>8</v>
       </c>
       <c r="J7" s="1"/>
-      <c r="K7" s="5"/>
+      <c r="K7" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="4"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="5"/>
       <c r="D8" s="1"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="2"/>
       <c r="G8" s="1"/>
       <c r="H8" s="2"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="5"/>
+      <c r="J8" s="8"/>
       <c r="K8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="3"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="2"/>
       <c r="G9" s="1"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="5"/>
+      <c r="I9" s="1"/>
       <c r="J9" s="1"/>
-      <c r="K9" s="8"/>
+      <c r="K9" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="4"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="1"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="F10" s="2"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="3"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="3"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="3"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="1"/>
       <c r="J11" s="4"/>
-      <c r="K11" s="8"/>
+      <c r="K11" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="9"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="9"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="3"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="8"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="3"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="8"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="3"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="3"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="8"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>